<commit_message>
Kosten, Qualität, Langfristplanung und Szenarien als Hypothesen
- Kostenmodell (kosten: Lektion, Räume je Typ, Schulhaus, Schulbus) und Qualitätskennzahlen
  als reine Auswertung des Ergebnisses; Optimierung bleibt unverändert (Schutztest)
- Langfristplanung als Kohortenmodell nach der Stufenfolge (Sek-Niveaus, Austritte,
  Wachstum, Quartierentwicklung) mit Klassen, fehlenden Räumen, Stellen und Kosten pro Jahr;
  behebt das Nachrücken nach Listenposition (S1C → S2A)
- Szenarien mit hypothese/ziel; App: Hypothesen über einfache Hebel anlegen, mehrere
  Szenarien rechnen und vergleichen, Reiter Planung & Kosten
- Eingaben für kosten/planung beim Einlesen geprüft; Bezüge in der Vorprüfung
- Python 3.10/3.11: f-Strings korrigiert, CI prüft die Syntax mit 3.10
- ergebnis.json/Schemas, Doku, Beispiel Malters, Screenshots aktualisiert

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DuTPgjhWjbXqkScDqKsY48
</commit_message>
<xml_diff>
--- a/beispiele/malters/ergebnis/Basis/stammdaten.xlsx
+++ b/beispiele/malters/ergebnis/Basis/stammdaten.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Foerderangebote'!$A$1:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Stundentafel'!$A$1:$L$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Kinder'!$A$1:$W$885</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Einstellungen'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Einstellungen'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -526,7 +526,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -918,19 +918,48 @@
           <t>planung</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>wachstum_prozent: 3</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>wachstum_prozent: 3
+vollpensum_lektionen: 28
+austritt_prozent:
+  '6': 10
+quartiere:
+- name: Neubaugebiet Nord
+  schulhaus: Bündtmättli
+  ab: 2029/30
+  wohnungen: 120
+  kinder_pro_wohnung: 0.3</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>kosten</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>annahme: Richtwerte für das Beispiel, nicht die Zahlen der Gemeinde Malters
+lektion_chf: 4000
+raum_chf:
+  Klassenzimmer: 15000
+  Kindergarten: 15000
+  Turnhalle: 45000
+  TTG-Zimmer: 12000
+schulhaus_chf: 90000
+transport_chf_pro_kind: 1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>gewichte</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>schulweg_pro_km: 100
 klasse: 400
@@ -939,7 +968,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>